<commit_message>
Sort of finished with ST accruals
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/CAST.ST.xlsx
+++ b/data/stx_xlsx/CAST.ST.xlsx
@@ -10184,7 +10184,10 @@
       <c r="O31" s="15">
         <v>31097.88</v>
       </c>
-      <c r="P31" s="15"/>
+      <c r="P31" s="15">
+        <f>SUM(P32:P33)</f>
+        <v>13.02</v>
+      </c>
       <c r="Q31" s="15">
         <v>27563.7</v>
       </c>
@@ -10206,7 +10209,10 @@
       <c r="W31" s="15">
         <v>17763.45</v>
       </c>
-      <c r="X31" s="15"/>
+      <c r="X31" s="15">
+        <f>SUM(X32:X33)</f>
+        <v>18.17</v>
+      </c>
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="14" t="s">

</xml_diff>